<commit_message>
feat: implement intelligent pristine board start detection filtering HUD and tutorial popups
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>00:22</t>
+          <t>00:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:36</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:18</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:06</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add Open Folder button on dashboard and update pristine level assets
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>00:24</t>
+          <t>00:22</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>00:36</t>
+          <t>00:38</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>05:20</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>08:18</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: pinpoint pristine board start via initial peak density & prevent image caching
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>00:22</t>
+          <t>00:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:44</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -581,7 +581,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:23</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:09</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: complete Game Design Deconstruction Suite with 5 specialized analyzers (SOLID) and multi-tab export
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Level_Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Level Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mechanics &amp; FTUE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Boosters &amp; Unlocks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pacing &amp; Difficulty" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Executive Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,28 +32,16 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,31 +55,14 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00E5E7EB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E5E7EB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E5E7EB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E5E7EB"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,262 +429,1163 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>Màn (Level)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Thời gian bắt đầu</t>
+          <t>Ảnh Khởi Đầu (Board Start)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Thời gian kết thúc</t>
+          <t>Ảnh Chiến Thắng (Victory / Reward)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Thời lượng giải (giây)</t>
+          <t>Thời Gian Bắt Đầu</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ảnh bắt đầu màn</t>
+          <t>Thời Gian Thắng</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ảnh chiến thắng</t>
+          <t>Thời Lượng Giải (s)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
+          <t>Độ Khó (Pacing)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ghi Chú Game Designer</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Level 01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>level_01/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>level_01/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>00:24</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>00:32</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="F2" t="n">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>level_01/board_start.jpg</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>level_01/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>🟢 Rất dễ (Tutorial)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Level 02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>level_02/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>level_02/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>00:44</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>02:51</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="F3" t="n">
         <v>126</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>level_02/board_start.jpg</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>level_02/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>🟡 Trung bình</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Level 03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>level_03/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>level_03/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>03:01</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>05:16</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="F4" t="n">
         <v>134</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>level_03/board_start.jpg</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>level_03/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>🟡 Trung bình</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Level 04</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>level_04/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>level_04/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>05:23</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>08:11</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="F5" t="n">
         <v>167</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>level_04/board_start.jpg</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>level_04/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>🔴 Khó (Thử thách)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Level 05</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>level_05/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>level_05/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>08:19</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>11:02</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="F6" t="n">
         <v>162</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>🔴 Khó (Thử thách)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Level 06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>level_06/board_start.jpg</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>level_06/victory.jpg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>181</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>🔴 Khó (Thử thách)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Màn (Level)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cơ Chế / Chướng Ngại Vật</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh Minh Họa Hướng Dẫn</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lời Thoại Hướng Dẫn (OCR)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Phân Loại FTUE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Quy Tắc Tương Tác</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tác Động Game Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Level 01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>🎮 Di Chuyển Cơ Bản (Core Match Mechanics)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>level_01/tutorial_ftue.jpg</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chạm cá đưa vào bình cùng loại để hoàn thành mục tiêu</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>🎯 Bắt buộc (Forced Tutorial)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Chọn cá trên bàn cờ di chuyển vào các bình rỗng phía trên</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FTUE làm quen luật chơi cốt lõi trong &lt; 10 giây, giảm thiểu Drop-off ngày đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Level 02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>🫧 Bong Bóng Khóa (Locked Bubble)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>level_02/tutorial_ftue.jpg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Whenbubblespop,new Tap anywhere to continue</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>🎯 Bắt buộc (Forced Tutorial - Bàn tay chỉ)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Thu thập đủ 3 cá cùng màu để giải phóng cá con bị giam bên trong</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Cơ chế giải đố phân tầng (Layered Goal), kích thích tò mò và cảm giác thỏa mãn khi nổ bóng</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Level 03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>level_03/tutorial_ftue.jpg</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Click on the adjacent fish three timesto defrosttheiceblock.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Level 04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>level_04/tutorial_ftue.jpg</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Click on the adjacent fish three times to defrost the ice block.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Level 05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>📈 Tăng Mật Độ &amp; Thử Thách (Board Density Scaling)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>level_05/board_start.jpg</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>level_05/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Không có hướng dẫn (Màn chơi tiêu chuẩn)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>👁️ Tự do (No Tutorial)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Tự do tính toán giải đố với bố cục mở rộng</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Thử thách kỹ năng người chơi với nhịp độ dồn dập hơn, chuẩn bị cho màn khó tiếp theo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Level 06</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>11:09</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>14:11</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>level_06/tutorial_ftue.jpg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Click on the adjacent fish three times to defrost the ice block.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tên Vật Phẩm / Tính Năng</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ảnh Icon Trợ Thủ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Màn Mở Khóa</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Thời Điểm Mở Khóa</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Phân Loại</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Công Dụng Cứu Nguy (Bailout Utility)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Đánh Giá Áp Lực Tiền Tệ (Monetization Pressure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>🏸 Vợt Bắt Cá (Net Booster)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>boosters/booster_net.jpg</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Level 03</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Level 03 (03:01)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>In-game Active Booster</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Thu thập ngay 1 nhóm cá bất kỳ mà không cần chờ bình rỗng. Cứu người chơi khi khay chờ sắp đầy.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>🟢 Áp lực thấp: Tặng miễn phí ở Lv.3 để kích thích thói quen dùng item (Habit Loop).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>🧹 Cây Cọ Quét (Clear Brush)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>boosters/booster_clear.jpg</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Level 05</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Level 05 (08:19)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Emergency Bailout Booster</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Quét dọn tức thời thanh chờ hoặc giải phóng 1 khối băng tắc nghẽn. Tránh bàn thua cận kề (Loss Aversion).</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>🟡 Áp lực trung bình: Giới thiệu ở Lv.5 khi các màn bắt đầu có 2 khối băng, bán gói cứu nguy ($0.99).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>🏺 Bình Cá Dự Phòng (Extra Jar Slot)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>boosters/booster_extra_slot.jpg</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Level 07</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Level 07 (Dự kiến mở khóa)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Permanent / Session Upgrade</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mở rộng không gian phân loại thêm 1 bình nước, giải tỏa áp lực sắp xếp cho các màn nhiều chủng loại cá.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>🔴 Áp lực cao: Mở khóa ở Lv.7, đây là điểm chốt chặn (Paywall) bán gói Starter Bundle hoặc xem Video Ads thưởng.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Màn (Level)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Thời Lượng Giải (s)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Độ Lệch Chuẩn (%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nhịp Độ Tâm Lý (Pacing Role)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Chỉ Số Căng Thẳng (Tension Tier)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nguy Cơ Bỏ Game (Choke Point Risk)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Khuyến Nghị Game Designer (Balancing Advice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Level 01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>🟢 Khởi Động (Tutorial / Warm-up)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1/5 (Thư giãn tuyệt đối)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>✅ Rất Thấp: FTUE dẫn dắt nhẹ nhàng</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Giữ nguyên luồng chơi, không nên tăng thêm chướng ngại vật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Level 02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>97%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>⚡ Đẩy Cao Trào (Tension Spike)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3.5/5 (Tập trung cao độ)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>🟡 Trung bình: Bắt đầu tạo áp lực phân vân</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Theo dõi thời gian suy nghĩ, kích thích người chơi nhìn vào thanh Booster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Level 03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>134</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>103%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>⚖️ Tiến Trình Tiêu Chuẩn (Steady Flow)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3/5 (Cân bằng)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅ An Toàn: Nhịp chơi ổn định</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Độ khó vừa vặn với kỹ năng người chơi tích lũy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Level 04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>167</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>129%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Level 05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>162</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>125%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Level 06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>181</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>level_06/board_start.jpg</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>level_06/victory.jpg</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>140%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Hạng Mục Phân Tích (Category)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Chỉ Số Thực Tế (Observed Metric)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Chuẩn Mực Casual/Puzzle (Industry Benchmark)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ý Nghĩa &amp; Khuyến Nghị Thực Chiến (Actionable Takeaway)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>⏱️ Quy Mô Phiên Chơi (Session Length)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12.9 phút (777s) cho 6 màn</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10 - 15 phút / session tiêu chuẩn cho Casual/Puzzle Mobile</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Thời lượng session lý tưởng để tiêu hao năng lượng (Energy loop) và kích hoạt quảng cáo Interstitial sau mỗi 2-3 màn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>⏳ Thời Lượng Trung Bình (Avg Level Duration)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>129.5 giây / màn (~2.2 phút)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>60s - 120s / level đối với game phân loại / match-3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Pacing chuẩn mực: người chơi có đủ thời gian tư duy mà không bị cảm giác lê thê kéo dài.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>🧩 Nhịp Giới Thiệu Cơ Chế (Novelty Pacing)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Màn 1 (Cơ bản) ➔ Màn 2 (Bong bóng) ➔ Màn 4 (Khối băng)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1 cơ chế mới mỗi 2-3 màn trong 10 màn đầu đời (D1 FTUE)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nhịp độ mở tính năng mới rất mượt: 2 màn đầu làm quen, màn 3 xả hơi, màn 4 thử thách thực sự.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>⚡ Hệ Thống Trợ Thủ (Booster Rollout)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mở khóa đều đặn: Lv.3 (Net) ➔ Lv.5 (Clear) ➔ Lv.7 (Slot)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mở khóa trước các màn thử thách để hình thành thói quen dùng item</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Chiến lược thông minh: Tặng Vợt ở Lv.3 ngay trước Màn 4 (màn khó đầu tiên), tạo thói quen dùng đồ giải cứu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>💰 Điểm Chạm Ép Nạp (Monetization Trigger Points)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Màn 4 (167s) và Màn 6 (181s) là hai điểm nghẽn (Choke Points)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Choke point xuất hiện ở màn 4-6 có tỷ lệ chuyển đổi nạp tiền cao nhất</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Vị trí vàng để pop-up gói ưu đãi Starter Bundle ($0.99) hoặc hiển thị nút 'Hồi Sinh / Thêm Nước Đi' giá 35 Coins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>💡 Đề Xuất Cải Tiến Cho Studio Của Mình</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Game đối thủ chưa có chuỗi thắng (Win Streak) và Pre-game Booster</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tính năng Win Streak (Royal Match) giúp tăng Retention D7 +15%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Studio nên bổ sung tính năng 'Chuỗi Thắng Bão Biển': Thắng liên tiếp sẽ được thả sẵn 1 bình cá thu thập trước khi vào màn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: split Mechanics Catalog and Level Curve Matrix, fix text wrapping in GAS v13, add SYSTEM_ARCHITECTURE_GUIDE and AGENTS rules
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Level Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mechanics &amp; FTUE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Boosters &amp; Unlocks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pacing &amp; Difficulty" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Executive Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Mechanics Catalog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Level Curve &amp; Mechanics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Boosters &amp; Unlocks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pacing &amp; Difficulty" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Executive Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -742,259 +743,247 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Màn (Level)</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cơ Chế / Chướng Ngại Vật</t>
+          <t>Mechanic Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Ảnh Minh Họa Hướng Dẫn</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Lời Thoại Hướng Dẫn (OCR)</t>
+          <t>Mô tả</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Phân Loại FTUE</t>
+          <t>Cách Hóa Giải / Tương Tác</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Quy Tắc Tương Tác</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Tác Động Game Design</t>
+          <t>Image_2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Level 01</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>🎮 Di Chuyển Cơ Bản (Core Match Mechanics)</t>
+          <t>Frozen Bubble</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>level_01/tutorial_ftue.jpg</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chạm cá đưa vào bình cùng loại để hoàn thành mục tiêu</t>
+          <t>Đóng băng toàn bộ bong bóng (mặc định là 3 nấc), không thể tương tác với cá bên trong.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🎯 Bắt buộc (Forced Tutorial)</t>
+          <t>Mỗi lần sort xong 1 bóng cá bất kỳ ở gần xung quanh sẽ giảm 1 nấc băng về 0 để mở bóng.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Chọn cá trên bàn cờ di chuyển vào các bình rỗng phía trên</t>
+          <t>level_04/board_start.jpg</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>FTUE làm quen luật chơi cốt lõi trong &lt; 10 giây, giảm thiểu Drop-off ngày đầu</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Level 02</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>🫧 Bong Bóng Khóa (Locked Bubble)</t>
+          <t>Bubble Lock &amp; Key</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>level_02/tutorial_ftue.jpg</t>
+          <t>Level 7</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Whenbubblespop,new Tap anywhere to continue</t>
+          <t>Khóa toàn bộ bong bóng, không thể lấy cá ra hoặc thả cá vào.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>🎯 Bắt buộc (Forced Tutorial - Bàn tay chỉ)</t>
+          <t>Thu thập Chìa khóa vàng (bubbleKey) ở bóng khác để tự động mở xích (hoặc dùng Búa).</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Thu thập đủ 3 cá cùng màu để giải phóng cá con bị giam bên trong</t>
+          <t>boosters/booster_net.jpg</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Cơ chế giải đố phân tầng (Layered Goal), kích thích tò mò và cảm giác thỏa mãn khi nổ bóng</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Level 03</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+          <t>Mystery Bubble</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>level_03/tutorial_ftue.jpg</t>
+          <t>Level 12</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Click on the adjacent fish three timesto defrosttheiceblock.</t>
+          <t>Sương mù che giấu hoàn toàn màu sắc và chủng loại của toàn bộ cá trong bóng.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+          <t>Tự động tan biến khi để bóng chạm đáy hoặc khi di chuyển đàn cá lân cận.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+          <t>boosters/booster_clear.jpg</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Level 04</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+          <t>Countdown Target Tank</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>level_04/tutorial_ftue.jpg</t>
+          <t>Level 20</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Click on the adjacent fish three times to defrost the ice block.</t>
+          <t>Bể mục tiêu có gắn đồng hồ đếm ngược thời gian thực, có chuông cảnh báo nhấp nháy đỏ.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+          <t>Bắt buộc phải ưu tiên gom đủ đàn cá cho bể này trước khi về 00:00, hết giờ sẽ thua Level.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+          <t>boosters/booster_extra_slot.jpg</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Level 05</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>📈 Tăng Mật Độ &amp; Thử Thách (Board Density Scaling)</t>
+          <t>Unknown Fish</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>level_05/board_start.jpg</t>
+          <t>Level 30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Không có hướng dẫn (Màn chơi tiêu chuẩn)</t>
+          <t>Con cá hiển thị dạng bóng đen có dấu hỏi (?), không thấy màu sắc thật khi nằm ở tầng dưới.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>👁️ Tự do (No Tutorial)</t>
+          <t>Là Hidden Fish, nhấn vào để chọn lên tầng trên thì mới hiện màu sắc thật của cá.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Tự do tính toán giải đố với bố cục mở rộng</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Thử thách kỹ năng người chơi với nhịp độ dồn dập hơn, chuẩn bị cho màn khó tiếp theo</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Level 06</t>
-        </is>
+      <c r="A7" t="n">
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>❄️ Khối Băng (Ice Block Obstacle)</t>
+          <t>Obstacle Stone</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>level_06/tutorial_ftue.jpg</t>
+          <t>Level 101</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Click on the adjacent fish three times to defrost the ice block.</t>
+          <t>Hòn đá ngầm chiếm slot cố định trong bóng, làm cản trở level, chiếm slot của các bóng khác.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>💡 Banner Gợi Ý Ngữ Cảnh (Contextual Tooltip)</t>
+          <t>Làm cản trở, chiếm diện tích trên level (Không thể clear được, phải sort né tránh).</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Click cá cùng màu lân cận 3 lần để rã đông khối băng</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Chướng ngại vật khóa ô, buộc người chơi gom nhóm xung quanh, tăng số nước đi và chiều sâu tính toán</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1009,155 +998,599 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tên Vật Phẩm / Tính Năng</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ảnh Icon Trợ Thủ</t>
+          <t>Level ID</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Màn Mở Khóa</t>
+          <t>Tier</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Thời Điểm Mở Khóa</t>
+          <t>BG ID</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Phân Loại</t>
+          <t>Mechanic_unlock</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Công Dụng Cứu Nguy (Bailout Utility)</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Đánh Giá Áp Lực Tiền Tệ (Monetization Pressure)</t>
+          <t>Bubble Type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Total Bubble Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Total_bubbles</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Fish_Type</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Fish_Type</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Fish</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Frozen Bubble</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Hidden Fish</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Foggy Bubble</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Locked Fish &amp; Key</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Lock &amp; Key Bubble</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Countdown Tank</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Bubble Spawner</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Reinforced Stone</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Frozen Fish</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Stone Obstacle</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>🏸 Vợt Bắt Cá (Net Booster)</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>boosters/booster_net.jpg</t>
+          <t>Lv.01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Level 03</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Level 03 (03:01)</t>
+          <t>BG_01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>In-game Active Booster</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Thu thập ngay 1 nhóm cá bất kỳ mà không cần chờ bình rỗng. Cứu người chơi khi khay chờ sắp đầy.</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>🟢 Áp lực thấp: Tặng miễn phí ở Lv.3 để kích thích thói quen dùng item (Habit Loop).</t>
-        </is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>17</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>49</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="b">
+        <v>0</v>
+      </c>
+      <c r="V2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>🧹 Cây Cọ Quét (Clear Brush)</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>boosters/booster_clear.jpg</t>
+          <t>Lv.02</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Level 05</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Level 05 (08:19)</t>
+          <t>BG_01</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Emergency Bailout Booster</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Quét dọn tức thời thanh chờ hoặc giải phóng 1 khối băng tắc nghẽn. Tránh bàn thua cận kề (Loss Aversion).</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>🟡 Áp lực trung bình: Giới thiệu ở Lv.5 khi các màn bắt đầu có 2 khối băng, bán gói cứu nguy ($0.99).</t>
-        </is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>22</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" t="n">
+        <v>62</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="b">
+        <v>0</v>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="b">
+        <v>0</v>
+      </c>
+      <c r="V3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>🏺 Bình Cá Dự Phòng (Extra Jar Slot)</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>boosters/booster_extra_slot.jpg</t>
+          <t>Lv.03</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Level 07</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Level 07 (Dự kiến mở khóa)</t>
+          <t>BG_01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Permanent / Session Upgrade</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mở rộng không gian phân loại thêm 1 bình nước, giải tỏa áp lực sắp xếp cho các màn nhiều chủng loại cá.</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>🔴 Áp lực cao: Mở khóa ở Lv.7, đây là điểm chốt chặn (Paywall) bán gói Starter Bundle hoặc xem Video Ads thưởng.</t>
-        </is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>27</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>75</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lv.04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Crazy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BG_02</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Frozen Bubble</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>32</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>88</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="U5" t="b">
+        <v>0</v>
+      </c>
+      <c r="V5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lv.05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Crazy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BG_02</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>37</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" t="n">
+        <v>101</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
+      </c>
+      <c r="U6" t="b">
+        <v>0</v>
+      </c>
+      <c r="V6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Lv.06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Crazy</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BG_02</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>42</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" t="n">
+        <v>114</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="U7" t="b">
+        <v>0</v>
+      </c>
+      <c r="V7" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1171,253 +1604,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Màn (Level)</t>
+          <t>Tên Vật Phẩm / Tính Năng</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Thời Lượng Giải (s)</t>
+          <t>Ảnh Icon Trợ Thủ</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Độ Lệch Chuẩn (%)</t>
+          <t>Màn Mở Khóa</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Nhịp Độ Tâm Lý (Pacing Role)</t>
+          <t>Thời Điểm Mở Khóa</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Chỉ Số Căng Thẳng (Tension Tier)</t>
+          <t>Phân Loại</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Nguy Cơ Bỏ Game (Choke Point Risk)</t>
+          <t>Công Dụng Cứu Nguy (Bailout Utility)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Khuyến Nghị Game Designer (Balancing Advice)</t>
+          <t>Đánh Giá Áp Lực Tiền Tệ (Monetization Pressure)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Level 01</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>7</v>
-      </c>
+          <t>🏸 Vợt Bắt Cá (Net Booster)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>Level 03</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>🟢 Khởi Động (Tutorial / Warm-up)</t>
+          <t>Màn 03</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1/5 (Thư giãn tuyệt đối)</t>
+          <t>In-game Active Booster</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>✅ Rất Thấp: FTUE dẫn dắt nhẹ nhàng</t>
+          <t>Thu thập ngay 1 nhóm cá bất kỳ mà không cần chờ bình rỗng. Cứu người chơi khi khay chờ sắp đầy.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Giữ nguyên luồng chơi, không nên tăng thêm chướng ngại vật.</t>
+          <t>🟢 Áp lực thấp: Tặng miễn phí ở Lv.3 để kích thích thói quen dùng item (Habit Loop).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Level 02</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>126</v>
-      </c>
+          <t>🧹 Cây Cọ Quét (Clear Brush)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>Level 05</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>⚡ Đẩy Cao Trào (Tension Spike)</t>
+          <t>Màn 05</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3.5/5 (Tập trung cao độ)</t>
+          <t>Emergency Bailout Booster</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>🟡 Trung bình: Bắt đầu tạo áp lực phân vân</t>
+          <t>Quét dọn tức thời thanh chờ hoặc giải phóng 1 khối băng tắc nghẽn. Tránh bàn thua cận kề (Loss Aversion).</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Theo dõi thời gian suy nghĩ, kích thích người chơi nhìn vào thanh Booster.</t>
+          <t>🟡 Áp lực trung bình: Giới thiệu ở Lv.5 khi các màn bắt đầu có 2 khối băng, bán gói cứu nguy ($0.99).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Level 03</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>134</v>
-      </c>
+          <t>🏺 Bình Cá Dự Phòng (Extra Jar Slot)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>103%</t>
+          <t>Level 07</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>⚖️ Tiến Trình Tiêu Chuẩn (Steady Flow)</t>
+          <t>Màn 07</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3/5 (Cân bằng)</t>
+          <t>Permanent / Session Upgrade</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>✅ An Toàn: Nhịp chơi ổn định</t>
+          <t>Mở rộng không gian phân loại thêm 1 bình nước, giải tỏa áp lực sắp xếp cho các màn nhiều chủng loại cá.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Độ khó vừa vặn với kỹ năng người chơi tích lũy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Level 04</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>167</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>129%</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>4.5/5 (Áp lực cao độ)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Level 05</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>162</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>125%</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>4.5/5 (Áp lực cao độ)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Level 06</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>181</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>140%</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>4.5/5 (Áp lực cao độ)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+          <t>🔴 Áp lực cao: Mở khóa ở Lv.7, đây là điểm chốt chặn (Paywall) bán gói Starter Bundle hoặc xem Video Ads thưởng.</t>
         </is>
       </c>
     </row>
@@ -1432,6 +1754,267 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Màn (Level)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Thời Lượng Giải (s)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Độ Lệch Chuẩn (%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Nhịp Độ Tâm Lý (Pacing Role)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Chỉ Số Căng Thẳng (Tension Tier)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nguy Cơ Bỏ Game (Choke Point Risk)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Khuyến Nghị Game Designer (Balancing Advice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Level 01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>🟢 Khởi Động (Tutorial / Warm-up)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1/5 (Thư giãn tuyệt đối)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>✅ Rất Thấp: FTUE dẫn dắt nhẹ nhàng</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Giữ nguyên luồng chơi, không nên tăng thêm chướng ngại vật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Level 02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>97%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>⚡ Đẩy Cao Trào (Tension Spike)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3.5/5 (Tập trung cao độ)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>🟡 Trung bình: Bắt đầu tạo áp lực phân vân</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Theo dõi thời gian suy nghĩ, kích thích người chơi nhìn vào thanh Booster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Level 03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>134</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>103%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>⚖️ Tiến Trình Tiêu Chuẩn (Steady Flow)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3/5 (Cân bằng)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅ An Toàn: Nhịp chơi ổn định</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Độ khó vừa vặn với kỹ năng người chơi tích lũy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Level 04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>167</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>129%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Level 05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>162</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>125%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Level 06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>181</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>140%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>🔥 Thử Thách Cực Hạn (Peak Challenge / Boss Feel)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4.5/5 (Áp lực cao độ)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>⚠️ NGUY CƠ CAO (Choke Point / Paywall)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Điểm ép nạp vật phẩm ($0.99) hoặc xem Ads hồi sinh. Cần tặng 1 Booster dùng thử trước đó.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
chore: update cached game_design_results and report.xlsx with clean booster and mechanic crops
</commit_message>
<xml_diff>
--- a/projects/FishSortPuzzle/report.xlsx
+++ b/projects/FishSortPuzzle/report.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>level_04/board_start.jpg</t>
+          <t>mechanics/mechanic_frozen_bubble.jpg</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>boosters/booster_net.jpg</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>boosters/booster_clear.jpg</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>boosters/booster_extra_slot.jpg</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1650,7 +1650,11 @@
           <t>🏸 Vợt Bắt Cá (Net Booster)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>boosters/booster_net.jpg</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Level 03</t>
@@ -1658,7 +1662,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Màn 03</t>
+          <t>03:01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1683,7 +1687,11 @@
           <t>🧹 Cây Cọ Quét (Clear Brush)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>boosters/booster_clear.jpg</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Level 05</t>
@@ -1691,7 +1699,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Màn 05</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1716,7 +1724,11 @@
           <t>🏺 Bình Cá Dự Phòng (Extra Jar Slot)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>boosters/booster_extra_slot.jpg</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Level 07</t>
@@ -1724,7 +1736,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Màn 07</t>
+          <t>Cuối video (Dự kiến)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>